<commit_message>
Việc 4.14: bỏ tính năng Luyện tập, đổi Thi thử -> Kiểm tra, Vấn đáp -> Tự luận
Bỏ hoàn toàn tính năng Luyện tập (backend: entity QuizResult/PracticeSet/
PracticeSetLopVisibility, endpoint, service; frontend: trang luyen-tap.html,
mọi nav-link, thẻ thống kê, cột trong các bảng xếp hạng). Field
Question.IsPublishedForPractice đổi tên thành IsPublished vì vẫn dùng để
publish/xóa Kiểm tra (Exam), không xóa.

Đổi hiển thị "Thi thử" -> "Kiểm tra" và "Vấn đáp" -> "Tự luận" xuyên suốt
frontend (tiêu đề, nhãn, toast, template Excel). Bỏ UI ghi âm/SpeechRecognition
ở trang thi-thu.html, chuyển sang nhập văn bản thuần cho phần Tự luận.
Entity OralQuestion/OralResult và EssayQuestion (chưa dùng) giữ nguyên.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/FrontEnd/template_cau_hoi.xlsx
+++ b/FrontEnd/template_cau_hoi.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CÂU HỎI" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="VẤN ĐÁP" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TỰ LUẬN" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -486,32 +486,32 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Chương 1: Cơ sở hình thành tư tưởng Hồ Chí Minh</t>
+          <t>Chương 1: (tên chương ví dụ)</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Tư tưởng Hồ Chí Minh được hình thành trên cơ sở nào sau đây?</t>
+          <t>Đây là câu hỏi trắc nghiệm mẫu — xóa dòng này và điền câu hỏi thật.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Chỉ chủ nghĩa Mác - Lênin</t>
+          <t>Lựa chọn A mẫu</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Truyền thống văn hóa dân tộc, tinh hoa văn hóa nhân loại và chủ nghĩa Mác - Lênin</t>
+          <t>Lựa chọn B mẫu</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Chỉ truyền thống văn hóa dân tộc</t>
+          <t>Lựa chọn C mẫu</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Chỉ tư tưởng phương Tây</t>
+          <t>Lựa chọn D mẫu</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -519,14 +519,14 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Tư tưởng Hồ Chí Minh là sự kết hợp giữa truyền thống dân tộc, tinh hoa nhân loại và chủ nghĩa Mác - Lênin, vận dụng sáng tạo vào điều kiện Việt Nam.</t>
+          <t>Giải thích mẫu cho đáp án đúng — điền lý do đáp án B (số 1) là đúng.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Chương 1: Cơ sở hình thành tư tưởng Hồ Chí Minh</t>
+          <t>Chương 1: (tên chương ví dụ)</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -591,7 +591,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Câu hỏi vấn đáp</t>
+          <t>Câu hỏi tự luận</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -608,17 +608,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Chương 1: Cơ sở hình thành tư tưởng Hồ Chí Minh</t>
+          <t>Chương 1: (tên chương ví dụ)</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Trình bày ngắn gọn 3 cơ sở hình thành tư tưởng Hồ Chí Minh.</t>
+          <t>Đây là câu hỏi tự luận mẫu — xóa dòng này và điền câu hỏi thật.</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Ba cơ sở: (1) truyền thống văn hóa, yêu nước của dân tộc Việt Nam; (2) tinh hoa văn hóa nhân loại (phương Đông và phương Tây); (3) chủ nghĩa Mác - Lênin — nhân tố quyết định bước phát triển về chất.</t>
+          <t>Đáp án chuẩn mẫu — điền nội dung đáp án tham khảo dùng để chấm điểm AI.</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -628,7 +628,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Chương 1: Cơ sở hình thành tư tưởng Hồ Chí Minh</t>
+          <t>Chương 1: (tên chương ví dụ)</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -638,7 +638,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>1 = dễ, 2 = trung bình, 3 = khó. Dùng để phân loại câu hỏi khi luyện tập vấn đáp.</t>
+          <t>1 = dễ, 2 = trung bình, 3 = khó. Dùng để phân loại câu hỏi khi luyện tập tự luận.</t>
         </is>
       </c>
       <c r="D3" t="n">

</xml_diff>